<commit_message>
feat: expand logistics operations and tracking
</commit_message>
<xml_diff>
--- a/docs/sample_material_import.xlsx
+++ b/docs/sample_material_import.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M.KELUAR" sheetId="1" r:id="R75de9eb602154ddb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M.KELUAR" sheetId="1" r:id="R518f73dc286d44ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -434,6 +434,7 @@
     <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -476,6 +477,9 @@
       <x:c r="M1" s="7" t="str">
         <x:v>TOKO/SUPPLIER</x:v>
       </x:c>
+      <x:c r="N1" t="str">
+        <x:v>KODE TRANSAKSI</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="9" t="n">
@@ -518,6 +522,9 @@
       <x:c r="M2" s="8" t="str">
         <x:v>CV. Sumber Bangunan</x:v>
       </x:c>
+      <x:c r="N2" t="str">
+        <x:v>MAT-IMP-001</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="9" t="n">
@@ -560,12 +567,51 @@
       <x:c r="M3" s="8" t="str">
         <x:v>TB. Maju Bersama</x:v>
       </x:c>
+      <x:c r="N3" t="str">
+        <x:v>MAT-IMP-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="N4"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="N5"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="N6"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="N7"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="N8"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="N9"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="N10"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="N11"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="N12"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="N13"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="N14"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="N15"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb18fe830d4d4349"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eeba2129e2a4cd9"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0aef956e822e4a8c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97c5aabea4c34cb5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>